<commit_message>
Atualiza compras pendentes 17/10/2026 22:01
</commit_message>
<xml_diff>
--- a/data/COMPRAS_PENDENTES.xlsx
+++ b/data/COMPRAS_PENDENTES.xlsx
@@ -2461,10 +2461,10 @@
     </row>
     <row r="74" customHeight="1" ht="20">
       <c r="A74" s="1" t="n">
-        <v>1607866</v>
+        <v>1604593</v>
       </c>
       <c r="B74" s="1" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C74" s="1" t="n">
         <v>9584</v>
@@ -2479,24 +2479,24 @@
         </is>
       </c>
       <c r="E74" s="1" t="n">
-        <v>1000</v>
+        <v>50</v>
       </c>
       <c r="F74" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">19/11/2026</t>
+            <t xml:space="preserve">20/01/2027</t>
           </r>
         </is>
       </c>
     </row>
     <row r="75" customHeight="1" ht="20">
       <c r="A75" s="1" t="n">
-        <v>1604593</v>
+        <v>1607866</v>
       </c>
       <c r="B75" s="1" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C75" s="1" t="n">
         <v>9584</v>
@@ -2511,14 +2511,14 @@
         </is>
       </c>
       <c r="E75" s="1" t="n">
-        <v>50</v>
+        <v>1000</v>
       </c>
       <c r="F75" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">20/01/2027</t>
+            <t xml:space="preserve">19/11/2026</t>
           </r>
         </is>
       </c>
@@ -15389,10 +15389,10 @@
     </row>
     <row r="478" customHeight="1" ht="20">
       <c r="A478" s="1" t="n">
-        <v>1523488</v>
+        <v>1587245</v>
       </c>
       <c r="B478" s="1" t="n">
-        <v>24896</v>
+        <v>27413</v>
       </c>
       <c r="C478" s="1" t="n">
         <v>14733</v>
@@ -15407,24 +15407,24 @@
         </is>
       </c>
       <c r="E478" s="1" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="F478" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">23/10/2026</t>
+            <t xml:space="preserve">26/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="479" customHeight="1" ht="20">
       <c r="A479" s="1" t="n">
-        <v>1587245</v>
+        <v>1523488</v>
       </c>
       <c r="B479" s="1" t="n">
-        <v>27413</v>
+        <v>24896</v>
       </c>
       <c r="C479" s="1" t="n">
         <v>14733</v>
@@ -15439,14 +15439,14 @@
         </is>
       </c>
       <c r="E479" s="1" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="F479" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">26/10/2026</t>
+            <t xml:space="preserve">23/10/2026</t>
           </r>
         </is>
       </c>

</xml_diff>

<commit_message>
Atualiza compras pendentes 18/10/2026 22:01
</commit_message>
<xml_diff>
--- a/data/COMPRAS_PENDENTES.xlsx
+++ b/data/COMPRAS_PENDENTES.xlsx
@@ -2461,10 +2461,10 @@
     </row>
     <row r="74" customHeight="1" ht="20">
       <c r="A74" s="1" t="n">
-        <v>1604593</v>
+        <v>1607866</v>
       </c>
       <c r="B74" s="1" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C74" s="1" t="n">
         <v>9584</v>
@@ -2479,24 +2479,24 @@
         </is>
       </c>
       <c r="E74" s="1" t="n">
-        <v>50</v>
+        <v>1000</v>
       </c>
       <c r="F74" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">20/01/2027</t>
+            <t xml:space="preserve">19/11/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="75" customHeight="1" ht="20">
       <c r="A75" s="1" t="n">
-        <v>1607866</v>
+        <v>1604593</v>
       </c>
       <c r="B75" s="1" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C75" s="1" t="n">
         <v>9584</v>
@@ -2511,14 +2511,14 @@
         </is>
       </c>
       <c r="E75" s="1" t="n">
-        <v>1000</v>
+        <v>50</v>
       </c>
       <c r="F75" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">19/11/2026</t>
+            <t xml:space="preserve">20/01/2027</t>
           </r>
         </is>
       </c>
@@ -7293,10 +7293,10 @@
     </row>
     <row r="225" customHeight="1" ht="20">
       <c r="A225" s="1" t="n">
-        <v>1542689</v>
+        <v>1470722</v>
       </c>
       <c r="B225" s="1" t="n">
-        <v>24951</v>
+        <v>24616</v>
       </c>
       <c r="C225" s="1" t="n">
         <v>10807</v>
@@ -7311,24 +7311,24 @@
         </is>
       </c>
       <c r="E225" s="1" t="n">
-        <v>3000</v>
+        <v>5000</v>
       </c>
       <c r="F225" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">23/11/2026</t>
+            <t xml:space="preserve">23/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="226" customHeight="1" ht="20">
       <c r="A226" s="1" t="n">
-        <v>1470722</v>
+        <v>1542689</v>
       </c>
       <c r="B226" s="1" t="n">
-        <v>24616</v>
+        <v>24951</v>
       </c>
       <c r="C226" s="1" t="n">
         <v>10807</v>
@@ -7343,14 +7343,14 @@
         </is>
       </c>
       <c r="E226" s="1" t="n">
-        <v>5000</v>
+        <v>3000</v>
       </c>
       <c r="F226" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">23/10/2026</t>
+            <t xml:space="preserve">23/11/2026</t>
           </r>
         </is>
       </c>
@@ -8029,10 +8029,10 @@
     </row>
     <row r="248" customHeight="1" ht="20">
       <c r="A248" s="1" t="n">
-        <v>1598892</v>
+        <v>1523488</v>
       </c>
       <c r="B248" s="1" t="n">
-        <v>27486</v>
+        <v>24896</v>
       </c>
       <c r="C248" s="1" t="n">
         <v>12593</v>
@@ -8047,24 +8047,24 @@
         </is>
       </c>
       <c r="E248" s="1" t="n">
-        <v>100</v>
+        <v>13</v>
       </c>
       <c r="F248" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/11/2026</t>
+            <t xml:space="preserve">23/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="249" customHeight="1" ht="20">
       <c r="A249" s="1" t="n">
-        <v>1523488</v>
+        <v>1598892</v>
       </c>
       <c r="B249" s="1" t="n">
-        <v>24896</v>
+        <v>27486</v>
       </c>
       <c r="C249" s="1" t="n">
         <v>12593</v>
@@ -8079,14 +8079,14 @@
         </is>
       </c>
       <c r="E249" s="1" t="n">
-        <v>13</v>
+        <v>100</v>
       </c>
       <c r="F249" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">23/10/2026</t>
+            <t xml:space="preserve">30/11/2026</t>
           </r>
         </is>
       </c>
@@ -10877,10 +10877,10 @@
     </row>
     <row r="337" customHeight="1" ht="20">
       <c r="A337" s="1" t="n">
-        <v>1598892</v>
+        <v>1523488</v>
       </c>
       <c r="B337" s="1" t="n">
-        <v>27486</v>
+        <v>24896</v>
       </c>
       <c r="C337" s="1" t="n">
         <v>13318</v>
@@ -10895,24 +10895,24 @@
         </is>
       </c>
       <c r="E337" s="1" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F337" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/11/2026</t>
+            <t xml:space="preserve">23/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="338" customHeight="1" ht="20">
       <c r="A338" s="1" t="n">
-        <v>1523488</v>
+        <v>1598892</v>
       </c>
       <c r="B338" s="1" t="n">
-        <v>24896</v>
+        <v>27486</v>
       </c>
       <c r="C338" s="1" t="n">
         <v>13318</v>
@@ -10927,14 +10927,14 @@
         </is>
       </c>
       <c r="E338" s="1" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F338" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">23/10/2026</t>
+            <t xml:space="preserve">30/11/2026</t>
           </r>
         </is>
       </c>
@@ -15261,10 +15261,10 @@
     </row>
     <row r="474" customHeight="1" ht="20">
       <c r="A474" s="1" t="n">
-        <v>1587245</v>
+        <v>1523488</v>
       </c>
       <c r="B474" s="1" t="n">
-        <v>27413</v>
+        <v>24896</v>
       </c>
       <c r="C474" s="1" t="n">
         <v>14730</v>
@@ -15279,24 +15279,24 @@
         </is>
       </c>
       <c r="E474" s="1" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="F474" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">26/10/2026</t>
+            <t xml:space="preserve">23/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="475" customHeight="1" ht="20">
       <c r="A475" s="1" t="n">
-        <v>1523488</v>
+        <v>1587245</v>
       </c>
       <c r="B475" s="1" t="n">
-        <v>24896</v>
+        <v>27413</v>
       </c>
       <c r="C475" s="1" t="n">
         <v>14730</v>
@@ -15311,14 +15311,14 @@
         </is>
       </c>
       <c r="E475" s="1" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="F475" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">23/10/2026</t>
+            <t xml:space="preserve">26/10/2026</t>
           </r>
         </is>
       </c>
@@ -15389,10 +15389,10 @@
     </row>
     <row r="478" customHeight="1" ht="20">
       <c r="A478" s="1" t="n">
-        <v>1587245</v>
+        <v>1523488</v>
       </c>
       <c r="B478" s="1" t="n">
-        <v>27413</v>
+        <v>24896</v>
       </c>
       <c r="C478" s="1" t="n">
         <v>14733</v>
@@ -15407,14 +15407,14 @@
         </is>
       </c>
       <c r="E478" s="1" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="F478" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">26/10/2026</t>
+            <t xml:space="preserve">23/10/2026</t>
           </r>
         </is>
       </c>
@@ -15453,10 +15453,10 @@
     </row>
     <row r="480" customHeight="1" ht="20">
       <c r="A480" s="1" t="n">
-        <v>1523488</v>
+        <v>1587245</v>
       </c>
       <c r="B480" s="1" t="n">
-        <v>24896</v>
+        <v>27413</v>
       </c>
       <c r="C480" s="1" t="n">
         <v>14733</v>
@@ -15471,14 +15471,14 @@
         </is>
       </c>
       <c r="E480" s="1" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="F480" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">23/10/2026</t>
+            <t xml:space="preserve">26/10/2026</t>
           </r>
         </is>
       </c>
@@ -31631,7 +31631,7 @@
         </is>
       </c>
       <c r="E985" s="1" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F985" s="1" t="inlineStr">
         <is>
@@ -31663,7 +31663,7 @@
         </is>
       </c>
       <c r="E986" s="1" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F986" s="1" t="inlineStr">
         <is>
@@ -37213,10 +37213,10 @@
     </row>
     <row r="1160" customHeight="1" ht="20">
       <c r="A1160" s="1" t="n">
-        <v>1587245</v>
+        <v>1523488</v>
       </c>
       <c r="B1160" s="1" t="n">
-        <v>27413</v>
+        <v>24896</v>
       </c>
       <c r="C1160" s="1" t="n">
         <v>31738</v>
@@ -37231,14 +37231,14 @@
         </is>
       </c>
       <c r="E1160" s="1" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="F1160" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">26/10/2026</t>
+            <t xml:space="preserve">23/10/2026</t>
           </r>
         </is>
       </c>
@@ -37277,10 +37277,10 @@
     </row>
     <row r="1162" customHeight="1" ht="20">
       <c r="A1162" s="1" t="n">
-        <v>1523488</v>
+        <v>1587245</v>
       </c>
       <c r="B1162" s="1" t="n">
-        <v>24896</v>
+        <v>27413</v>
       </c>
       <c r="C1162" s="1" t="n">
         <v>31738</v>
@@ -37295,14 +37295,14 @@
         </is>
       </c>
       <c r="E1162" s="1" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="F1162" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">23/10/2026</t>
+            <t xml:space="preserve">26/10/2026</t>
           </r>
         </is>
       </c>
@@ -37437,10 +37437,10 @@
     </row>
     <row r="1167" customHeight="1" ht="20">
       <c r="A1167" s="1" t="n">
-        <v>1587245</v>
+        <v>1523488</v>
       </c>
       <c r="B1167" s="1" t="n">
-        <v>27413</v>
+        <v>24896</v>
       </c>
       <c r="C1167" s="1" t="n">
         <v>31737</v>
@@ -37455,24 +37455,24 @@
         </is>
       </c>
       <c r="E1167" s="1" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="F1167" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">26/10/2026</t>
+            <t xml:space="preserve">23/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1168" customHeight="1" ht="20">
       <c r="A1168" s="1" t="n">
-        <v>1523488</v>
+        <v>1587245</v>
       </c>
       <c r="B1168" s="1" t="n">
-        <v>24896</v>
+        <v>27413</v>
       </c>
       <c r="C1168" s="1" t="n">
         <v>31737</v>
@@ -37487,14 +37487,14 @@
         </is>
       </c>
       <c r="E1168" s="1" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="F1168" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">23/10/2026</t>
+            <t xml:space="preserve">26/10/2026</t>
           </r>
         </is>
       </c>
@@ -39741,10 +39741,10 @@
     </row>
     <row r="1239" customHeight="1" ht="20">
       <c r="A1239" s="1" t="n">
-        <v>1598892</v>
+        <v>1523488</v>
       </c>
       <c r="B1239" s="1" t="n">
-        <v>27486</v>
+        <v>24896</v>
       </c>
       <c r="C1239" s="1" t="n">
         <v>33659</v>
@@ -39759,24 +39759,24 @@
         </is>
       </c>
       <c r="E1239" s="1" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F1239" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/11/2026</t>
+            <t xml:space="preserve">23/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1240" customHeight="1" ht="20">
       <c r="A1240" s="1" t="n">
-        <v>1523488</v>
+        <v>1598892</v>
       </c>
       <c r="B1240" s="1" t="n">
-        <v>24896</v>
+        <v>27486</v>
       </c>
       <c r="C1240" s="1" t="n">
         <v>33659</v>
@@ -39791,14 +39791,14 @@
         </is>
       </c>
       <c r="E1240" s="1" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F1240" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">23/10/2026</t>
+            <t xml:space="preserve">30/11/2026</t>
           </r>
         </is>
       </c>
@@ -43645,10 +43645,10 @@
     </row>
     <row r="1361" customHeight="1" ht="20">
       <c r="A1361" s="1" t="n">
-        <v>1598892</v>
+        <v>1523488</v>
       </c>
       <c r="B1361" s="1" t="n">
-        <v>27486</v>
+        <v>24896</v>
       </c>
       <c r="C1361" s="1" t="n">
         <v>37934</v>
@@ -43663,24 +43663,24 @@
         </is>
       </c>
       <c r="E1361" s="1" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F1361" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/11/2026</t>
+            <t xml:space="preserve">23/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1362" customHeight="1" ht="20">
       <c r="A1362" s="1" t="n">
-        <v>1523488</v>
+        <v>1598892</v>
       </c>
       <c r="B1362" s="1" t="n">
-        <v>24896</v>
+        <v>27486</v>
       </c>
       <c r="C1362" s="1" t="n">
         <v>37934</v>
@@ -43695,14 +43695,14 @@
         </is>
       </c>
       <c r="E1362" s="1" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F1362" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">23/10/2026</t>
+            <t xml:space="preserve">30/11/2026</t>
           </r>
         </is>
       </c>
@@ -43773,10 +43773,10 @@
     </row>
     <row r="1365" customHeight="1" ht="20">
       <c r="A1365" s="1" t="n">
-        <v>1598892</v>
+        <v>1523488</v>
       </c>
       <c r="B1365" s="1" t="n">
-        <v>27486</v>
+        <v>24896</v>
       </c>
       <c r="C1365" s="1" t="n">
         <v>39413</v>
@@ -43791,24 +43791,24 @@
         </is>
       </c>
       <c r="E1365" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1365" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/11/2026</t>
+            <t xml:space="preserve">23/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1366" customHeight="1" ht="20">
       <c r="A1366" s="1" t="n">
-        <v>1523488</v>
+        <v>1598892</v>
       </c>
       <c r="B1366" s="1" t="n">
-        <v>24896</v>
+        <v>27486</v>
       </c>
       <c r="C1366" s="1" t="n">
         <v>39413</v>
@@ -43823,14 +43823,14 @@
         </is>
       </c>
       <c r="E1366" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F1366" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">23/10/2026</t>
+            <t xml:space="preserve">30/11/2026</t>
           </r>
         </is>
       </c>
@@ -48125,10 +48125,10 @@
     </row>
     <row r="1501" customHeight="1" ht="20">
       <c r="A1501" s="1" t="n">
-        <v>1624906</v>
+        <v>1598892</v>
       </c>
       <c r="B1501" s="1" t="n">
-        <v>29565</v>
+        <v>27486</v>
       </c>
       <c r="C1501" s="1" t="n">
         <v>43440</v>
@@ -48143,24 +48143,24 @@
         </is>
       </c>
       <c r="E1501" s="1" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="F1501" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">08/11/2026</t>
+            <t xml:space="preserve">30/11/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1502" customHeight="1" ht="20">
       <c r="A1502" s="1" t="n">
-        <v>1598892</v>
+        <v>1624906</v>
       </c>
       <c r="B1502" s="1" t="n">
-        <v>27486</v>
+        <v>29565</v>
       </c>
       <c r="C1502" s="1" t="n">
         <v>43440</v>
@@ -48175,14 +48175,14 @@
         </is>
       </c>
       <c r="E1502" s="1" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="F1502" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/11/2026</t>
+            <t xml:space="preserve">08/11/2026</t>
           </r>
         </is>
       </c>
@@ -48445,10 +48445,10 @@
     </row>
     <row r="1511" customHeight="1" ht="20">
       <c r="A1511" s="1" t="n">
-        <v>1624906</v>
+        <v>1598892</v>
       </c>
       <c r="B1511" s="1" t="n">
-        <v>29565</v>
+        <v>27486</v>
       </c>
       <c r="C1511" s="1" t="n">
         <v>43441</v>
@@ -48463,14 +48463,14 @@
         </is>
       </c>
       <c r="E1511" s="1" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="F1511" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">08/11/2026</t>
+            <t xml:space="preserve">30/11/2026</t>
           </r>
         </is>
       </c>
@@ -48495,7 +48495,7 @@
         </is>
       </c>
       <c r="E1512" s="1" t="n">
-        <v>150</v>
+        <v>1</v>
       </c>
       <c r="F1512" s="1" t="inlineStr">
         <is>
@@ -48509,10 +48509,10 @@
     </row>
     <row r="1513" customHeight="1" ht="20">
       <c r="A1513" s="1" t="n">
-        <v>1598892</v>
+        <v>1624906</v>
       </c>
       <c r="B1513" s="1" t="n">
-        <v>27486</v>
+        <v>29565</v>
       </c>
       <c r="C1513" s="1" t="n">
         <v>43441</v>
@@ -48527,14 +48527,14 @@
         </is>
       </c>
       <c r="E1513" s="1" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="F1513" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/11/2026</t>
+            <t xml:space="preserve">08/11/2026</t>
           </r>
         </is>
       </c>
@@ -48701,10 +48701,10 @@
     </row>
     <row r="1519" customHeight="1" ht="20">
       <c r="A1519" s="1" t="n">
-        <v>1598892</v>
+        <v>1523488</v>
       </c>
       <c r="B1519" s="1" t="n">
-        <v>27486</v>
+        <v>24896</v>
       </c>
       <c r="C1519" s="1" t="n">
         <v>44178</v>
@@ -48726,17 +48726,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/11/2026</t>
+            <t xml:space="preserve">23/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1520" customHeight="1" ht="20">
       <c r="A1520" s="1" t="n">
-        <v>1523488</v>
+        <v>1598892</v>
       </c>
       <c r="B1520" s="1" t="n">
-        <v>24896</v>
+        <v>27486</v>
       </c>
       <c r="C1520" s="1" t="n">
         <v>44178</v>
@@ -48758,7 +48758,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">23/10/2026</t>
+            <t xml:space="preserve">30/11/2026</t>
           </r>
         </is>
       </c>
@@ -49085,10 +49085,10 @@
     </row>
     <row r="1531" customHeight="1" ht="20">
       <c r="A1531" s="1" t="n">
-        <v>1598892</v>
+        <v>1523488</v>
       </c>
       <c r="B1531" s="1" t="n">
-        <v>27486</v>
+        <v>24896</v>
       </c>
       <c r="C1531" s="1" t="n">
         <v>44087</v>
@@ -49103,24 +49103,24 @@
         </is>
       </c>
       <c r="E1531" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1531" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/11/2026</t>
+            <t xml:space="preserve">23/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1532" customHeight="1" ht="20">
       <c r="A1532" s="1" t="n">
-        <v>1523488</v>
+        <v>1598892</v>
       </c>
       <c r="B1532" s="1" t="n">
-        <v>24896</v>
+        <v>27486</v>
       </c>
       <c r="C1532" s="1" t="n">
         <v>44087</v>
@@ -49135,14 +49135,14 @@
         </is>
       </c>
       <c r="E1532" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F1532" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">23/10/2026</t>
+            <t xml:space="preserve">30/11/2026</t>
           </r>
         </is>
       </c>
@@ -49693,10 +49693,10 @@
     </row>
     <row r="1550" customHeight="1" ht="20">
       <c r="A1550" s="1" t="n">
-        <v>1624906</v>
+        <v>1598892</v>
       </c>
       <c r="B1550" s="1" t="n">
-        <v>29565</v>
+        <v>27486</v>
       </c>
       <c r="C1550" s="1" t="n">
         <v>43437</v>
@@ -49711,24 +49711,24 @@
         </is>
       </c>
       <c r="E1550" s="1" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="F1550" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">08/11/2026</t>
+            <t xml:space="preserve">30/11/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1551" customHeight="1" ht="20">
       <c r="A1551" s="1" t="n">
-        <v>1598892</v>
+        <v>1624906</v>
       </c>
       <c r="B1551" s="1" t="n">
-        <v>27486</v>
+        <v>29565</v>
       </c>
       <c r="C1551" s="1" t="n">
         <v>43437</v>
@@ -49743,14 +49743,14 @@
         </is>
       </c>
       <c r="E1551" s="1" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="F1551" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/11/2026</t>
+            <t xml:space="preserve">08/11/2026</t>
           </r>
         </is>
       </c>

</xml_diff>

<commit_message>
Atualiza compras pendentes 24/10/2026 22:01
</commit_message>
<xml_diff>
--- a/data/COMPRAS_PENDENTES.xlsx
+++ b/data/COMPRAS_PENDENTES.xlsx
@@ -4829,10 +4829,10 @@
     </row>
     <row r="148" customHeight="1" ht="20">
       <c r="A148" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B148" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C148" s="1" t="n">
         <v>9411</v>
@@ -4847,24 +4847,24 @@
         </is>
       </c>
       <c r="E148" s="1" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="F148" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="149" customHeight="1" ht="20">
       <c r="A149" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B149" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C149" s="1" t="n">
         <v>9411</v>
@@ -4879,14 +4879,14 @@
         </is>
       </c>
       <c r="E149" s="1" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="F149" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -5277,10 +5277,10 @@
     </row>
     <row r="162" customHeight="1" ht="20">
       <c r="A162" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B162" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C162" s="1" t="n">
         <v>9418</v>
@@ -5295,24 +5295,24 @@
         </is>
       </c>
       <c r="E162" s="1" t="n">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="F162" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="163" customHeight="1" ht="20">
       <c r="A163" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B163" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C163" s="1" t="n">
         <v>9418</v>
@@ -5327,14 +5327,14 @@
         </is>
       </c>
       <c r="E163" s="1" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="F163" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -5501,10 +5501,10 @@
     </row>
     <row r="169" customHeight="1" ht="20">
       <c r="A169" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B169" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C169" s="1" t="n">
         <v>9423</v>
@@ -5526,17 +5526,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="170" customHeight="1" ht="20">
       <c r="A170" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B170" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C170" s="1" t="n">
         <v>9423</v>
@@ -5558,7 +5558,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -6717,10 +6717,10 @@
     </row>
     <row r="207" customHeight="1" ht="20">
       <c r="A207" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B207" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C207" s="1" t="n">
         <v>11311</v>
@@ -6742,17 +6742,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="208" customHeight="1" ht="20">
       <c r="A208" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B208" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C208" s="1" t="n">
         <v>11311</v>
@@ -6774,7 +6774,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -11837,10 +11837,10 @@
     </row>
     <row r="367" customHeight="1" ht="20">
       <c r="A367" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B367" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C367" s="1" t="n">
         <v>13665</v>
@@ -11855,24 +11855,24 @@
         </is>
       </c>
       <c r="E367" s="1" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="F367" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="368" customHeight="1" ht="20">
       <c r="A368" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B368" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C368" s="1" t="n">
         <v>13665</v>
@@ -11887,14 +11887,14 @@
         </is>
       </c>
       <c r="E368" s="1" t="n">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="F368" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -12029,10 +12029,10 @@
     </row>
     <row r="373" customHeight="1" ht="20">
       <c r="A373" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B373" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C373" s="1" t="n">
         <v>13761</v>
@@ -12047,24 +12047,24 @@
         </is>
       </c>
       <c r="E373" s="1" t="n">
-        <v>3000</v>
+        <v>200</v>
       </c>
       <c r="F373" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="374" customHeight="1" ht="20">
       <c r="A374" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B374" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C374" s="1" t="n">
         <v>13761</v>
@@ -12079,14 +12079,14 @@
         </is>
       </c>
       <c r="E374" s="1" t="n">
-        <v>200</v>
+        <v>3000</v>
       </c>
       <c r="F374" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -12797,10 +12797,10 @@
     </row>
     <row r="397" customHeight="1" ht="20">
       <c r="A397" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B397" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C397" s="1" t="n">
         <v>13763</v>
@@ -12815,24 +12815,24 @@
         </is>
       </c>
       <c r="E397" s="1" t="n">
-        <v>2000</v>
+        <v>300</v>
       </c>
       <c r="F397" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="398" customHeight="1" ht="20">
       <c r="A398" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B398" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C398" s="1" t="n">
         <v>13763</v>
@@ -12847,24 +12847,24 @@
         </is>
       </c>
       <c r="E398" s="1" t="n">
-        <v>300</v>
+        <v>2000</v>
       </c>
       <c r="F398" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
     </row>
     <row r="399" customHeight="1" ht="20">
       <c r="A399" s="1" t="n">
-        <v>1630636</v>
+        <v>1523488</v>
       </c>
       <c r="B399" s="1" t="n">
-        <v>29656</v>
+        <v>24896</v>
       </c>
       <c r="C399" s="1" t="n">
         <v>13766</v>
@@ -12879,24 +12879,24 @@
         </is>
       </c>
       <c r="E399" s="1" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="F399" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">26/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="400" customHeight="1" ht="20">
       <c r="A400" s="1" t="n">
-        <v>1523488</v>
+        <v>1630636</v>
       </c>
       <c r="B400" s="1" t="n">
-        <v>24896</v>
+        <v>29656</v>
       </c>
       <c r="C400" s="1" t="n">
         <v>13766</v>
@@ -12911,14 +12911,14 @@
         </is>
       </c>
       <c r="E400" s="1" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="F400" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">26/10/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -13309,10 +13309,10 @@
     </row>
     <row r="413" customHeight="1" ht="20">
       <c r="A413" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B413" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C413" s="1" t="n">
         <v>13185</v>
@@ -13327,24 +13327,24 @@
         </is>
       </c>
       <c r="E413" s="1" t="n">
-        <v>3000</v>
+        <v>300</v>
       </c>
       <c r="F413" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="414" customHeight="1" ht="20">
       <c r="A414" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B414" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C414" s="1" t="n">
         <v>13185</v>
@@ -13359,14 +13359,14 @@
         </is>
       </c>
       <c r="E414" s="1" t="n">
-        <v>300</v>
+        <v>3000</v>
       </c>
       <c r="F414" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -13725,10 +13725,10 @@
     </row>
     <row r="426" customHeight="1" ht="20">
       <c r="A426" s="1" t="n">
-        <v>1598892</v>
+        <v>1523488</v>
       </c>
       <c r="B426" s="1" t="n">
-        <v>27486</v>
+        <v>24896</v>
       </c>
       <c r="C426" s="1" t="n">
         <v>13939</v>
@@ -13743,24 +13743,24 @@
         </is>
       </c>
       <c r="E426" s="1" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F426" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">26/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="427" customHeight="1" ht="20">
       <c r="A427" s="1" t="n">
-        <v>1523488</v>
+        <v>1598892</v>
       </c>
       <c r="B427" s="1" t="n">
-        <v>24896</v>
+        <v>27486</v>
       </c>
       <c r="C427" s="1" t="n">
         <v>13939</v>
@@ -13775,14 +13775,14 @@
         </is>
       </c>
       <c r="E427" s="1" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F427" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">26/10/2026</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
@@ -15197,10 +15197,10 @@
     </row>
     <row r="472" customHeight="1" ht="20">
       <c r="A472" s="1" t="n">
-        <v>1630636</v>
+        <v>1523488</v>
       </c>
       <c r="B472" s="1" t="n">
-        <v>29656</v>
+        <v>24896</v>
       </c>
       <c r="C472" s="1" t="n">
         <v>13503</v>
@@ -15222,17 +15222,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">26/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="473" customHeight="1" ht="20">
       <c r="A473" s="1" t="n">
-        <v>1523488</v>
+        <v>1630636</v>
       </c>
       <c r="B473" s="1" t="n">
-        <v>24896</v>
+        <v>29656</v>
       </c>
       <c r="C473" s="1" t="n">
         <v>13503</v>
@@ -15254,7 +15254,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">26/10/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -15453,10 +15453,10 @@
     </row>
     <row r="480" customHeight="1" ht="20">
       <c r="A480" s="1" t="n">
-        <v>1630636</v>
+        <v>1523488</v>
       </c>
       <c r="B480" s="1" t="n">
-        <v>29656</v>
+        <v>24896</v>
       </c>
       <c r="C480" s="1" t="n">
         <v>13507</v>
@@ -15471,24 +15471,24 @@
         </is>
       </c>
       <c r="E480" s="1" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F480" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">26/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="481" customHeight="1" ht="20">
       <c r="A481" s="1" t="n">
-        <v>1523488</v>
+        <v>1630636</v>
       </c>
       <c r="B481" s="1" t="n">
-        <v>24896</v>
+        <v>29656</v>
       </c>
       <c r="C481" s="1" t="n">
         <v>13507</v>
@@ -15503,24 +15503,24 @@
         </is>
       </c>
       <c r="E481" s="1" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F481" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">26/10/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
     </row>
     <row r="482" customHeight="1" ht="20">
       <c r="A482" s="1" t="n">
-        <v>1630636</v>
+        <v>1523488</v>
       </c>
       <c r="B482" s="1" t="n">
-        <v>29656</v>
+        <v>24896</v>
       </c>
       <c r="C482" s="1" t="n">
         <v>13508</v>
@@ -15535,24 +15535,24 @@
         </is>
       </c>
       <c r="E482" s="1" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F482" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">26/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="483" customHeight="1" ht="20">
       <c r="A483" s="1" t="n">
-        <v>1523488</v>
+        <v>1630636</v>
       </c>
       <c r="B483" s="1" t="n">
-        <v>24896</v>
+        <v>29656</v>
       </c>
       <c r="C483" s="1" t="n">
         <v>13508</v>
@@ -15567,14 +15567,14 @@
         </is>
       </c>
       <c r="E483" s="1" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F483" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">26/10/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -15677,10 +15677,10 @@
     </row>
     <row r="487" customHeight="1" ht="20">
       <c r="A487" s="1" t="n">
-        <v>1630636</v>
+        <v>1523488</v>
       </c>
       <c r="B487" s="1" t="n">
-        <v>29656</v>
+        <v>24896</v>
       </c>
       <c r="C487" s="1" t="n">
         <v>13510</v>
@@ -15702,17 +15702,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">26/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="488" customHeight="1" ht="20">
       <c r="A488" s="1" t="n">
-        <v>1523488</v>
+        <v>1630636</v>
       </c>
       <c r="B488" s="1" t="n">
-        <v>24896</v>
+        <v>29656</v>
       </c>
       <c r="C488" s="1" t="n">
         <v>13510</v>
@@ -15734,7 +15734,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">26/10/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -16541,10 +16541,10 @@
     </row>
     <row r="514" customHeight="1" ht="20">
       <c r="A514" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B514" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C514" s="1" t="n">
         <v>13182</v>
@@ -16566,17 +16566,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="515" customHeight="1" ht="20">
       <c r="A515" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B515" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C515" s="1" t="n">
         <v>13182</v>
@@ -16598,7 +16598,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -16957,10 +16957,10 @@
     </row>
     <row r="527" customHeight="1" ht="20">
       <c r="A527" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B527" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C527" s="1" t="n">
         <v>13764</v>
@@ -16975,24 +16975,24 @@
         </is>
       </c>
       <c r="E527" s="1" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="F527" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="528" customHeight="1" ht="20">
       <c r="A528" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B528" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C528" s="1" t="n">
         <v>13764</v>
@@ -17007,24 +17007,24 @@
         </is>
       </c>
       <c r="E528" s="1" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="F528" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
     </row>
     <row r="529" customHeight="1" ht="20">
       <c r="A529" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B529" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C529" s="1" t="n">
         <v>13765</v>
@@ -17046,17 +17046,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="530" customHeight="1" ht="20">
       <c r="A530" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B530" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C530" s="1" t="n">
         <v>13765</v>
@@ -17078,7 +17078,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -17117,10 +17117,10 @@
     </row>
     <row r="532" customHeight="1" ht="20">
       <c r="A532" s="1" t="n">
-        <v>1630636</v>
+        <v>1523488</v>
       </c>
       <c r="B532" s="1" t="n">
-        <v>29656</v>
+        <v>24896</v>
       </c>
       <c r="C532" s="1" t="n">
         <v>13770</v>
@@ -17135,24 +17135,24 @@
         </is>
       </c>
       <c r="E532" s="1" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F532" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">26/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="533" customHeight="1" ht="20">
       <c r="A533" s="1" t="n">
-        <v>1523488</v>
+        <v>1630636</v>
       </c>
       <c r="B533" s="1" t="n">
-        <v>24896</v>
+        <v>29656</v>
       </c>
       <c r="C533" s="1" t="n">
         <v>13770</v>
@@ -17167,14 +17167,14 @@
         </is>
       </c>
       <c r="E533" s="1" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F533" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">26/10/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -17629,10 +17629,10 @@
     </row>
     <row r="548" customHeight="1" ht="20">
       <c r="A548" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B548" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C548" s="1" t="n">
         <v>13437</v>
@@ -17654,17 +17654,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="549" customHeight="1" ht="20">
       <c r="A549" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B549" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C549" s="1" t="n">
         <v>13437</v>
@@ -17686,7 +17686,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -17725,10 +17725,10 @@
     </row>
     <row r="551" customHeight="1" ht="20">
       <c r="A551" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B551" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C551" s="1" t="n">
         <v>13664</v>
@@ -17750,17 +17750,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="552" customHeight="1" ht="20">
       <c r="A552" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B552" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C552" s="1" t="n">
         <v>13664</v>
@@ -17782,7 +17782,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -18237,10 +18237,10 @@
     </row>
     <row r="567" customHeight="1" ht="20">
       <c r="A567" s="1" t="n">
-        <v>1630636</v>
+        <v>1523488</v>
       </c>
       <c r="B567" s="1" t="n">
-        <v>29656</v>
+        <v>24896</v>
       </c>
       <c r="C567" s="1" t="n">
         <v>13449</v>
@@ -18262,17 +18262,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">26/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="568" customHeight="1" ht="20">
       <c r="A568" s="1" t="n">
-        <v>1523488</v>
+        <v>1630636</v>
       </c>
       <c r="B568" s="1" t="n">
-        <v>24896</v>
+        <v>29656</v>
       </c>
       <c r="C568" s="1" t="n">
         <v>13449</v>
@@ -18294,7 +18294,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">26/10/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -18653,10 +18653,10 @@
     </row>
     <row r="580" customHeight="1" ht="20">
       <c r="A580" s="1" t="n">
-        <v>1630636</v>
+        <v>1523488</v>
       </c>
       <c r="B580" s="1" t="n">
-        <v>29656</v>
+        <v>24896</v>
       </c>
       <c r="C580" s="1" t="n">
         <v>14218</v>
@@ -18678,17 +18678,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">26/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="581" customHeight="1" ht="20">
       <c r="A581" s="1" t="n">
-        <v>1523488</v>
+        <v>1630636</v>
       </c>
       <c r="B581" s="1" t="n">
-        <v>24896</v>
+        <v>29656</v>
       </c>
       <c r="C581" s="1" t="n">
         <v>14218</v>
@@ -18710,7 +18710,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">26/10/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -18941,10 +18941,10 @@
     </row>
     <row r="589" customHeight="1" ht="20">
       <c r="A589" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B589" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C589" s="1" t="n">
         <v>14811</v>
@@ -18959,24 +18959,24 @@
         </is>
       </c>
       <c r="E589" s="1" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="F589" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="590" customHeight="1" ht="20">
       <c r="A590" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B590" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C590" s="1" t="n">
         <v>14811</v>
@@ -18991,24 +18991,24 @@
         </is>
       </c>
       <c r="E590" s="1" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="F590" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
     </row>
     <row r="591" customHeight="1" ht="20">
       <c r="A591" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B591" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C591" s="1" t="n">
         <v>14843</v>
@@ -19023,24 +19023,24 @@
         </is>
       </c>
       <c r="E591" s="1" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="F591" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="592" customHeight="1" ht="20">
       <c r="A592" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B592" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C592" s="1" t="n">
         <v>14843</v>
@@ -19055,14 +19055,14 @@
         </is>
       </c>
       <c r="E592" s="1" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="F592" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -19325,10 +19325,10 @@
     </row>
     <row r="601" customHeight="1" ht="20">
       <c r="A601" s="1" t="n">
-        <v>1598892</v>
+        <v>1523488</v>
       </c>
       <c r="B601" s="1" t="n">
-        <v>27486</v>
+        <v>24896</v>
       </c>
       <c r="C601" s="1" t="n">
         <v>14791</v>
@@ -19350,17 +19350,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">26/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="602" customHeight="1" ht="20">
       <c r="A602" s="1" t="n">
-        <v>1523488</v>
+        <v>1598892</v>
       </c>
       <c r="B602" s="1" t="n">
-        <v>24896</v>
+        <v>27486</v>
       </c>
       <c r="C602" s="1" t="n">
         <v>14791</v>
@@ -19382,7 +19382,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">26/10/2026</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
@@ -19549,10 +19549,10 @@
     </row>
     <row r="608" customHeight="1" ht="20">
       <c r="A608" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B608" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C608" s="1" t="n">
         <v>14986</v>
@@ -19574,17 +19574,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="609" customHeight="1" ht="20">
       <c r="A609" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B609" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C609" s="1" t="n">
         <v>14986</v>
@@ -19606,7 +19606,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -19997,10 +19997,10 @@
     </row>
     <row r="622" customHeight="1" ht="20">
       <c r="A622" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B622" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C622" s="1" t="n">
         <v>14491</v>
@@ -20015,24 +20015,24 @@
         </is>
       </c>
       <c r="E622" s="1" t="n">
-        <v>5000</v>
+        <v>10000</v>
       </c>
       <c r="F622" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="623" customHeight="1" ht="20">
       <c r="A623" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B623" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C623" s="1" t="n">
         <v>14491</v>
@@ -20047,14 +20047,14 @@
         </is>
       </c>
       <c r="E623" s="1" t="n">
-        <v>10000</v>
+        <v>5000</v>
       </c>
       <c r="F623" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -20253,10 +20253,10 @@
     </row>
     <row r="630" customHeight="1" ht="20">
       <c r="A630" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B630" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C630" s="1" t="n">
         <v>14495</v>
@@ -20271,24 +20271,24 @@
         </is>
       </c>
       <c r="E630" s="1" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="F630" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="631" customHeight="1" ht="20">
       <c r="A631" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B631" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C631" s="1" t="n">
         <v>14495</v>
@@ -20303,14 +20303,14 @@
         </is>
       </c>
       <c r="E631" s="1" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="F631" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -21053,10 +21053,10 @@
     </row>
     <row r="655" customHeight="1" ht="20">
       <c r="A655" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B655" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C655" s="1" t="n">
         <v>14494</v>
@@ -21078,17 +21078,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="656" customHeight="1" ht="20">
       <c r="A656" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B656" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C656" s="1" t="n">
         <v>14494</v>
@@ -21110,7 +21110,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -21661,10 +21661,10 @@
     </row>
     <row r="674" customHeight="1" ht="20">
       <c r="A674" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B674" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C674" s="1" t="n">
         <v>14493</v>
@@ -21679,24 +21679,24 @@
         </is>
       </c>
       <c r="E674" s="1" t="n">
-        <v>5000</v>
+        <v>10000</v>
       </c>
       <c r="F674" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="675" customHeight="1" ht="20">
       <c r="A675" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B675" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C675" s="1" t="n">
         <v>14493</v>
@@ -21711,14 +21711,14 @@
         </is>
       </c>
       <c r="E675" s="1" t="n">
-        <v>10000</v>
+        <v>5000</v>
       </c>
       <c r="F675" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -21981,10 +21981,10 @@
     </row>
     <row r="684" customHeight="1" ht="20">
       <c r="A684" s="1" t="n">
-        <v>1635939</v>
+        <v>1598892</v>
       </c>
       <c r="B684" s="1" t="n">
-        <v>29609</v>
+        <v>27486</v>
       </c>
       <c r="C684" s="1" t="n">
         <v>14137</v>
@@ -21999,24 +21999,24 @@
         </is>
       </c>
       <c r="E684" s="1" t="n">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="F684" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">13/11/2026</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="685" customHeight="1" ht="20">
       <c r="A685" s="1" t="n">
-        <v>1598892</v>
+        <v>1635939</v>
       </c>
       <c r="B685" s="1" t="n">
-        <v>27486</v>
+        <v>29609</v>
       </c>
       <c r="C685" s="1" t="n">
         <v>14137</v>
@@ -22031,14 +22031,14 @@
         </is>
       </c>
       <c r="E685" s="1" t="n">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="F685" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">13/11/2026</t>
           </r>
         </is>
       </c>
@@ -23069,10 +23069,10 @@
     </row>
     <row r="718" customHeight="1" ht="20">
       <c r="A718" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B718" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C718" s="1" t="n">
         <v>15498</v>
@@ -23087,24 +23087,24 @@
         </is>
       </c>
       <c r="E718" s="1" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F718" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="719" customHeight="1" ht="20">
       <c r="A719" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B719" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C719" s="1" t="n">
         <v>15498</v>
@@ -23119,24 +23119,24 @@
         </is>
       </c>
       <c r="E719" s="1" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F719" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
     </row>
     <row r="720" customHeight="1" ht="20">
       <c r="A720" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B720" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C720" s="1" t="n">
         <v>15499</v>
@@ -23151,24 +23151,24 @@
         </is>
       </c>
       <c r="E720" s="1" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="F720" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="721" customHeight="1" ht="20">
       <c r="A721" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B721" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C721" s="1" t="n">
         <v>15499</v>
@@ -23183,14 +23183,14 @@
         </is>
       </c>
       <c r="E721" s="1" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="F721" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -23741,10 +23741,10 @@
     </row>
     <row r="739" customHeight="1" ht="20">
       <c r="A739" s="1" t="n">
-        <v>1630636</v>
+        <v>1523488</v>
       </c>
       <c r="B739" s="1" t="n">
-        <v>29656</v>
+        <v>24896</v>
       </c>
       <c r="C739" s="1" t="n">
         <v>15479</v>
@@ -23759,24 +23759,24 @@
         </is>
       </c>
       <c r="E739" s="1" t="n">
-        <v>500</v>
+        <v>50</v>
       </c>
       <c r="F739" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">26/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="740" customHeight="1" ht="20">
       <c r="A740" s="1" t="n">
-        <v>1523488</v>
+        <v>1598892</v>
       </c>
       <c r="B740" s="1" t="n">
-        <v>24896</v>
+        <v>27486</v>
       </c>
       <c r="C740" s="1" t="n">
         <v>15479</v>
@@ -23791,24 +23791,24 @@
         </is>
       </c>
       <c r="E740" s="1" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="F740" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">26/10/2026</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="741" customHeight="1" ht="20">
       <c r="A741" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B741" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C741" s="1" t="n">
         <v>15479</v>
@@ -23823,14 +23823,14 @@
         </is>
       </c>
       <c r="E741" s="1" t="n">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="F741" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -23869,10 +23869,10 @@
     </row>
     <row r="743" customHeight="1" ht="20">
       <c r="A743" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B743" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C743" s="1" t="n">
         <v>15864</v>
@@ -23887,24 +23887,24 @@
         </is>
       </c>
       <c r="E743" s="1" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="F743" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="744" customHeight="1" ht="20">
       <c r="A744" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B744" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C744" s="1" t="n">
         <v>15864</v>
@@ -23919,14 +23919,14 @@
         </is>
       </c>
       <c r="E744" s="1" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="F744" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -24029,10 +24029,10 @@
     </row>
     <row r="748" customHeight="1" ht="20">
       <c r="A748" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B748" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C748" s="1" t="n">
         <v>15485</v>
@@ -24047,24 +24047,24 @@
         </is>
       </c>
       <c r="E748" s="1" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F748" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="749" customHeight="1" ht="20">
       <c r="A749" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B749" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C749" s="1" t="n">
         <v>15485</v>
@@ -24079,14 +24079,14 @@
         </is>
       </c>
       <c r="E749" s="1" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F749" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -24349,10 +24349,10 @@
     </row>
     <row r="758" customHeight="1" ht="20">
       <c r="A758" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B758" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C758" s="1" t="n">
         <v>15507</v>
@@ -24367,14 +24367,14 @@
         </is>
       </c>
       <c r="E758" s="1" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="F758" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
@@ -24399,7 +24399,7 @@
         </is>
       </c>
       <c r="E759" s="1" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F759" s="1" t="inlineStr">
         <is>
@@ -24413,10 +24413,10 @@
     </row>
     <row r="760" customHeight="1" ht="20">
       <c r="A760" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B760" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C760" s="1" t="n">
         <v>15507</v>
@@ -24431,14 +24431,14 @@
         </is>
       </c>
       <c r="E760" s="1" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="F760" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -24477,10 +24477,10 @@
     </row>
     <row r="762" customHeight="1" ht="20">
       <c r="A762" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B762" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C762" s="1" t="n">
         <v>15484</v>
@@ -24495,24 +24495,24 @@
         </is>
       </c>
       <c r="E762" s="1" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="F762" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="763" customHeight="1" ht="20">
       <c r="A763" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B763" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C763" s="1" t="n">
         <v>15484</v>
@@ -24527,14 +24527,14 @@
         </is>
       </c>
       <c r="E763" s="1" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="F763" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -24669,10 +24669,10 @@
     </row>
     <row r="768" customHeight="1" ht="20">
       <c r="A768" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B768" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C768" s="1" t="n">
         <v>15377</v>
@@ -24687,24 +24687,24 @@
         </is>
       </c>
       <c r="E768" s="1" t="n">
-        <v>5000</v>
+        <v>3000</v>
       </c>
       <c r="F768" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="769" customHeight="1" ht="20">
       <c r="A769" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B769" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C769" s="1" t="n">
         <v>15377</v>
@@ -24719,14 +24719,14 @@
         </is>
       </c>
       <c r="E769" s="1" t="n">
-        <v>3000</v>
+        <v>5000</v>
       </c>
       <c r="F769" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -24797,10 +24797,10 @@
     </row>
     <row r="772" customHeight="1" ht="20">
       <c r="A772" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B772" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C772" s="1" t="n">
         <v>15178</v>
@@ -24822,17 +24822,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="773" customHeight="1" ht="20">
       <c r="A773" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B773" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C773" s="1" t="n">
         <v>15178</v>
@@ -24854,7 +24854,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -24957,10 +24957,10 @@
     </row>
     <row r="777" customHeight="1" ht="20">
       <c r="A777" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B777" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C777" s="1" t="n">
         <v>15505</v>
@@ -24975,14 +24975,14 @@
         </is>
       </c>
       <c r="E777" s="1" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F777" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
@@ -25007,7 +25007,7 @@
         </is>
       </c>
       <c r="E778" s="1" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F778" s="1" t="inlineStr">
         <is>
@@ -25021,10 +25021,10 @@
     </row>
     <row r="779" customHeight="1" ht="20">
       <c r="A779" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B779" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C779" s="1" t="n">
         <v>15505</v>
@@ -25039,14 +25039,14 @@
         </is>
       </c>
       <c r="E779" s="1" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F779" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -25309,10 +25309,10 @@
     </row>
     <row r="788" customHeight="1" ht="20">
       <c r="A788" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B788" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C788" s="1" t="n">
         <v>15378</v>
@@ -25327,24 +25327,24 @@
         </is>
       </c>
       <c r="E788" s="1" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="F788" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="789" customHeight="1" ht="20">
       <c r="A789" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B789" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C789" s="1" t="n">
         <v>15378</v>
@@ -25359,14 +25359,14 @@
         </is>
       </c>
       <c r="E789" s="1" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="F789" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -25437,10 +25437,10 @@
     </row>
     <row r="792" customHeight="1" ht="20">
       <c r="A792" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B792" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C792" s="1" t="n">
         <v>15660</v>
@@ -25462,17 +25462,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="793" customHeight="1" ht="20">
       <c r="A793" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B793" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C793" s="1" t="n">
         <v>15660</v>
@@ -25494,7 +25494,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -25533,10 +25533,10 @@
     </row>
     <row r="795" customHeight="1" ht="20">
       <c r="A795" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B795" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C795" s="1" t="n">
         <v>15662</v>
@@ -25558,17 +25558,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="796" customHeight="1" ht="20">
       <c r="A796" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B796" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C796" s="1" t="n">
         <v>15662</v>
@@ -25590,7 +25590,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -26045,10 +26045,10 @@
     </row>
     <row r="811" customHeight="1" ht="20">
       <c r="A811" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B811" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C811" s="1" t="n">
         <v>15867</v>
@@ -26070,17 +26070,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="812" customHeight="1" ht="20">
       <c r="A812" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B812" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C812" s="1" t="n">
         <v>15867</v>
@@ -26102,7 +26102,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -26301,10 +26301,10 @@
     </row>
     <row r="819" customHeight="1" ht="20">
       <c r="A819" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B819" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C819" s="1" t="n">
         <v>15856</v>
@@ -26326,17 +26326,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="820" customHeight="1" ht="20">
       <c r="A820" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B820" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C820" s="1" t="n">
         <v>15856</v>
@@ -26358,7 +26358,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -26461,10 +26461,10 @@
     </row>
     <row r="824" customHeight="1" ht="20">
       <c r="A824" s="1" t="n">
-        <v>1630636</v>
+        <v>1523488</v>
       </c>
       <c r="B824" s="1" t="n">
-        <v>29656</v>
+        <v>24896</v>
       </c>
       <c r="C824" s="1" t="n">
         <v>15183</v>
@@ -26479,24 +26479,24 @@
         </is>
       </c>
       <c r="E824" s="1" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="F824" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">26/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="825" customHeight="1" ht="20">
       <c r="A825" s="1" t="n">
-        <v>1523488</v>
+        <v>1598892</v>
       </c>
       <c r="B825" s="1" t="n">
-        <v>24896</v>
+        <v>27486</v>
       </c>
       <c r="C825" s="1" t="n">
         <v>15183</v>
@@ -26511,24 +26511,24 @@
         </is>
       </c>
       <c r="E825" s="1" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F825" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">26/10/2026</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="826" customHeight="1" ht="20">
       <c r="A826" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B826" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C826" s="1" t="n">
         <v>15183</v>
@@ -26543,14 +26543,14 @@
         </is>
       </c>
       <c r="E826" s="1" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="F826" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -26781,10 +26781,10 @@
     </row>
     <row r="834" customHeight="1" ht="20">
       <c r="A834" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B834" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C834" s="1" t="n">
         <v>15376</v>
@@ -26799,24 +26799,24 @@
         </is>
       </c>
       <c r="E834" s="1" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="F834" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="835" customHeight="1" ht="20">
       <c r="A835" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B835" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C835" s="1" t="n">
         <v>15376</v>
@@ -26831,14 +26831,14 @@
         </is>
       </c>
       <c r="E835" s="1" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="F835" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -27421,10 +27421,10 @@
     </row>
     <row r="854" customHeight="1" ht="20">
       <c r="A854" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B854" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C854" s="1" t="n">
         <v>24866</v>
@@ -27446,17 +27446,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="855" customHeight="1" ht="20">
       <c r="A855" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B855" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C855" s="1" t="n">
         <v>24866</v>
@@ -27478,7 +27478,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -27581,10 +27581,10 @@
     </row>
     <row r="859" customHeight="1" ht="20">
       <c r="A859" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B859" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C859" s="1" t="n">
         <v>24865</v>
@@ -27606,17 +27606,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="860" customHeight="1" ht="20">
       <c r="A860" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B860" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C860" s="1" t="n">
         <v>24865</v>
@@ -27638,7 +27638,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -28669,10 +28669,10 @@
     </row>
     <row r="893" customHeight="1" ht="20">
       <c r="A893" s="1" t="n">
-        <v>1598892</v>
+        <v>1523488</v>
       </c>
       <c r="B893" s="1" t="n">
-        <v>27486</v>
+        <v>24896</v>
       </c>
       <c r="C893" s="1" t="n">
         <v>25879</v>
@@ -28687,24 +28687,24 @@
         </is>
       </c>
       <c r="E893" s="1" t="n">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="F893" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">26/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="894" customHeight="1" ht="20">
       <c r="A894" s="1" t="n">
-        <v>1523488</v>
+        <v>1598892</v>
       </c>
       <c r="B894" s="1" t="n">
-        <v>24896</v>
+        <v>27486</v>
       </c>
       <c r="C894" s="1" t="n">
         <v>25879</v>
@@ -28719,14 +28719,14 @@
         </is>
       </c>
       <c r="E894" s="1" t="n">
-        <v>600</v>
+        <v>500</v>
       </c>
       <c r="F894" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">26/10/2026</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
@@ -29181,10 +29181,10 @@
     </row>
     <row r="909" customHeight="1" ht="20">
       <c r="A909" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B909" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C909" s="1" t="n">
         <v>26413</v>
@@ -29199,24 +29199,24 @@
         </is>
       </c>
       <c r="E909" s="1" t="n">
-        <v>3000</v>
+        <v>2000</v>
       </c>
       <c r="F909" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="910" customHeight="1" ht="20">
       <c r="A910" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B910" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C910" s="1" t="n">
         <v>26413</v>
@@ -29231,24 +29231,24 @@
         </is>
       </c>
       <c r="E910" s="1" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="F910" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
     </row>
     <row r="911" customHeight="1" ht="20">
       <c r="A911" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B911" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C911" s="1" t="n">
         <v>26414</v>
@@ -29270,17 +29270,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="912" customHeight="1" ht="20">
       <c r="A912" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B912" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C912" s="1" t="n">
         <v>26414</v>
@@ -29302,7 +29302,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -29373,10 +29373,10 @@
     </row>
     <row r="915" customHeight="1" ht="20">
       <c r="A915" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B915" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C915" s="1" t="n">
         <v>26417</v>
@@ -29398,17 +29398,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="916" customHeight="1" ht="20">
       <c r="A916" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B916" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C916" s="1" t="n">
         <v>26417</v>
@@ -29430,7 +29430,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -30429,10 +30429,10 @@
     </row>
     <row r="948" customHeight="1" ht="20">
       <c r="A948" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B948" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C948" s="1" t="n">
         <v>26083</v>
@@ -30454,17 +30454,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="949" customHeight="1" ht="20">
       <c r="A949" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B949" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C949" s="1" t="n">
         <v>26083</v>
@@ -30486,7 +30486,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -30621,10 +30621,10 @@
     </row>
     <row r="954" customHeight="1" ht="20">
       <c r="A954" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B954" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C954" s="1" t="n">
         <v>26474</v>
@@ -30639,24 +30639,24 @@
         </is>
       </c>
       <c r="E954" s="1" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="F954" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="955" customHeight="1" ht="20">
       <c r="A955" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B955" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C955" s="1" t="n">
         <v>26474</v>
@@ -30671,24 +30671,24 @@
         </is>
       </c>
       <c r="E955" s="1" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="F955" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
     </row>
     <row r="956" customHeight="1" ht="20">
       <c r="A956" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B956" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C956" s="1" t="n">
         <v>26475</v>
@@ -30703,24 +30703,24 @@
         </is>
       </c>
       <c r="E956" s="1" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="F956" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="957" customHeight="1" ht="20">
       <c r="A957" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B957" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C957" s="1" t="n">
         <v>26475</v>
@@ -30735,14 +30735,14 @@
         </is>
       </c>
       <c r="E957" s="1" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="F957" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -30941,10 +30941,10 @@
     </row>
     <row r="964" customHeight="1" ht="20">
       <c r="A964" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B964" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C964" s="1" t="n">
         <v>26479</v>
@@ -30966,17 +30966,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="965" customHeight="1" ht="20">
       <c r="A965" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B965" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C965" s="1" t="n">
         <v>26479</v>
@@ -30998,7 +30998,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -31453,10 +31453,10 @@
     </row>
     <row r="980" customHeight="1" ht="20">
       <c r="A980" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B980" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C980" s="1" t="n">
         <v>26497</v>
@@ -31471,24 +31471,24 @@
         </is>
       </c>
       <c r="E980" s="1" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="F980" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="981" customHeight="1" ht="20">
       <c r="A981" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B981" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C981" s="1" t="n">
         <v>26497</v>
@@ -31503,14 +31503,14 @@
         </is>
       </c>
       <c r="E981" s="1" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="F981" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -31549,10 +31549,10 @@
     </row>
     <row r="983" customHeight="1" ht="20">
       <c r="A983" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B983" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C983" s="1" t="n">
         <v>26501</v>
@@ -31567,24 +31567,24 @@
         </is>
       </c>
       <c r="E983" s="1" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F983" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="984" customHeight="1" ht="20">
       <c r="A984" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B984" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C984" s="1" t="n">
         <v>26501</v>
@@ -31599,14 +31599,14 @@
         </is>
       </c>
       <c r="E984" s="1" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F984" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -33117,10 +33117,10 @@
     </row>
     <row r="1032" customHeight="1" ht="20">
       <c r="A1032" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B1032" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C1032" s="1" t="n">
         <v>26469</v>
@@ -33142,17 +33142,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1033" customHeight="1" ht="20">
       <c r="A1033" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B1033" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C1033" s="1" t="n">
         <v>26469</v>
@@ -33174,7 +33174,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -35293,10 +35293,10 @@
     </row>
     <row r="1100" customHeight="1" ht="20">
       <c r="A1100" s="1" t="n">
-        <v>1630636</v>
+        <v>1523488</v>
       </c>
       <c r="B1100" s="1" t="n">
-        <v>29656</v>
+        <v>24896</v>
       </c>
       <c r="C1100" s="1" t="n">
         <v>26539</v>
@@ -35311,24 +35311,24 @@
         </is>
       </c>
       <c r="E1100" s="1" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="F1100" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">26/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1101" customHeight="1" ht="20">
       <c r="A1101" s="1" t="n">
-        <v>1523488</v>
+        <v>1630636</v>
       </c>
       <c r="B1101" s="1" t="n">
-        <v>24896</v>
+        <v>29656</v>
       </c>
       <c r="C1101" s="1" t="n">
         <v>26539</v>
@@ -35343,14 +35343,14 @@
         </is>
       </c>
       <c r="E1101" s="1" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="F1101" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">26/10/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -35421,10 +35421,10 @@
     </row>
     <row r="1104" customHeight="1" ht="20">
       <c r="A1104" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B1104" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C1104" s="1" t="n">
         <v>26503</v>
@@ -35446,17 +35446,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1105" customHeight="1" ht="20">
       <c r="A1105" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B1105" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C1105" s="1" t="n">
         <v>26503</v>
@@ -35478,7 +35478,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -35517,10 +35517,10 @@
     </row>
     <row r="1107" customHeight="1" ht="20">
       <c r="A1107" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B1107" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C1107" s="1" t="n">
         <v>26504</v>
@@ -35535,24 +35535,24 @@
         </is>
       </c>
       <c r="E1107" s="1" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="F1107" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1108" customHeight="1" ht="20">
       <c r="A1108" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B1108" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C1108" s="1" t="n">
         <v>26504</v>
@@ -35567,14 +35567,14 @@
         </is>
       </c>
       <c r="E1108" s="1" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="F1108" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -35677,10 +35677,10 @@
     </row>
     <row r="1112" customHeight="1" ht="20">
       <c r="A1112" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B1112" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C1112" s="1" t="n">
         <v>26508</v>
@@ -35702,17 +35702,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1113" customHeight="1" ht="20">
       <c r="A1113" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B1113" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C1113" s="1" t="n">
         <v>26508</v>
@@ -35734,7 +35734,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -35997,10 +35997,10 @@
     </row>
     <row r="1122" customHeight="1" ht="20">
       <c r="A1122" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B1122" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C1122" s="1" t="n">
         <v>27415</v>
@@ -36022,17 +36022,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1123" customHeight="1" ht="20">
       <c r="A1123" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B1123" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C1123" s="1" t="n">
         <v>27415</v>
@@ -36054,7 +36054,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -36797,10 +36797,10 @@
     </row>
     <row r="1147" customHeight="1" ht="20">
       <c r="A1147" s="1" t="n">
-        <v>1630636</v>
+        <v>1523488</v>
       </c>
       <c r="B1147" s="1" t="n">
-        <v>29656</v>
+        <v>24896</v>
       </c>
       <c r="C1147" s="1" t="n">
         <v>27413</v>
@@ -36815,24 +36815,24 @@
         </is>
       </c>
       <c r="E1147" s="1" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="F1147" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">26/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1148" customHeight="1" ht="20">
       <c r="A1148" s="1" t="n">
-        <v>1523488</v>
+        <v>1598892</v>
       </c>
       <c r="B1148" s="1" t="n">
-        <v>24896</v>
+        <v>27486</v>
       </c>
       <c r="C1148" s="1" t="n">
         <v>27413</v>
@@ -36847,24 +36847,24 @@
         </is>
       </c>
       <c r="E1148" s="1" t="n">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="F1148" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">26/10/2026</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1149" customHeight="1" ht="20">
       <c r="A1149" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B1149" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C1149" s="1" t="n">
         <v>27413</v>
@@ -36886,7 +36886,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -37181,10 +37181,10 @@
     </row>
     <row r="1159" customHeight="1" ht="20">
       <c r="A1159" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B1159" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C1159" s="1" t="n">
         <v>27646</v>
@@ -37199,24 +37199,24 @@
         </is>
       </c>
       <c r="E1159" s="1" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="F1159" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1160" customHeight="1" ht="20">
       <c r="A1160" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B1160" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C1160" s="1" t="n">
         <v>27646</v>
@@ -37231,14 +37231,14 @@
         </is>
       </c>
       <c r="E1160" s="1" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="F1160" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -37533,10 +37533,10 @@
     </row>
     <row r="1170" customHeight="1" ht="20">
       <c r="A1170" s="1" t="n">
-        <v>1598892</v>
+        <v>1523488</v>
       </c>
       <c r="B1170" s="1" t="n">
-        <v>27486</v>
+        <v>24896</v>
       </c>
       <c r="C1170" s="1" t="n">
         <v>27756</v>
@@ -37551,24 +37551,24 @@
         </is>
       </c>
       <c r="E1170" s="1" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="F1170" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">26/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1171" customHeight="1" ht="20">
       <c r="A1171" s="1" t="n">
-        <v>1523488</v>
+        <v>1598892</v>
       </c>
       <c r="B1171" s="1" t="n">
-        <v>24896</v>
+        <v>27486</v>
       </c>
       <c r="C1171" s="1" t="n">
         <v>27756</v>
@@ -37583,14 +37583,14 @@
         </is>
       </c>
       <c r="E1171" s="1" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="F1171" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">26/10/2026</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
@@ -40687,7 +40687,7 @@
         </is>
       </c>
       <c r="E1268" s="1" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F1268" s="1" t="inlineStr">
         <is>
@@ -40719,7 +40719,7 @@
         </is>
       </c>
       <c r="E1269" s="1" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F1269" s="1" t="inlineStr">
         <is>
@@ -47325,10 +47325,10 @@
     </row>
     <row r="1476" customHeight="1" ht="20">
       <c r="A1476" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B1476" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C1476" s="1" t="n">
         <v>31114</v>
@@ -47343,24 +47343,24 @@
         </is>
       </c>
       <c r="E1476" s="1" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F1476" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1477" customHeight="1" ht="20">
       <c r="A1477" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B1477" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C1477" s="1" t="n">
         <v>31114</v>
@@ -47375,14 +47375,14 @@
         </is>
       </c>
       <c r="E1477" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F1477" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -48605,10 +48605,10 @@
     </row>
     <row r="1516" customHeight="1" ht="20">
       <c r="A1516" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B1516" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C1516" s="1" t="n">
         <v>32987</v>
@@ -48630,17 +48630,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1517" customHeight="1" ht="20">
       <c r="A1517" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B1517" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C1517" s="1" t="n">
         <v>32987</v>
@@ -48662,7 +48662,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -48861,10 +48861,10 @@
     </row>
     <row r="1524" customHeight="1" ht="20">
       <c r="A1524" s="1" t="n">
-        <v>1630636</v>
+        <v>1523488</v>
       </c>
       <c r="B1524" s="1" t="n">
-        <v>29656</v>
+        <v>24896</v>
       </c>
       <c r="C1524" s="1" t="n">
         <v>32696</v>
@@ -48886,17 +48886,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">26/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1525" customHeight="1" ht="20">
       <c r="A1525" s="1" t="n">
-        <v>1523488</v>
+        <v>1630636</v>
       </c>
       <c r="B1525" s="1" t="n">
-        <v>24896</v>
+        <v>29656</v>
       </c>
       <c r="C1525" s="1" t="n">
         <v>32696</v>
@@ -48918,7 +48918,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">26/10/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -52765,10 +52765,10 @@
     </row>
     <row r="1646" customHeight="1" ht="20">
       <c r="A1646" s="1" t="n">
-        <v>1598892</v>
+        <v>1523488</v>
       </c>
       <c r="B1646" s="1" t="n">
-        <v>27486</v>
+        <v>24896</v>
       </c>
       <c r="C1646" s="1" t="n">
         <v>37398</v>
@@ -52790,17 +52790,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">26/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1647" customHeight="1" ht="20">
       <c r="A1647" s="1" t="n">
-        <v>1523488</v>
+        <v>1598892</v>
       </c>
       <c r="B1647" s="1" t="n">
-        <v>24896</v>
+        <v>27486</v>
       </c>
       <c r="C1647" s="1" t="n">
         <v>37398</v>
@@ -52822,7 +52822,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">26/10/2026</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
@@ -54461,10 +54461,10 @@
     </row>
     <row r="1699" customHeight="1" ht="20">
       <c r="A1699" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B1699" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C1699" s="1" t="n">
         <v>39295</v>
@@ -54479,24 +54479,24 @@
         </is>
       </c>
       <c r="E1699" s="1" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F1699" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1700" customHeight="1" ht="20">
       <c r="A1700" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B1700" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C1700" s="1" t="n">
         <v>39295</v>
@@ -54511,14 +54511,14 @@
         </is>
       </c>
       <c r="E1700" s="1" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F1700" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -54973,10 +54973,10 @@
     </row>
     <row r="1715" customHeight="1" ht="20">
       <c r="A1715" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B1715" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C1715" s="1" t="n">
         <v>39299</v>
@@ -54991,24 +54991,24 @@
         </is>
       </c>
       <c r="E1715" s="1" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="F1715" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1716" customHeight="1" ht="20">
       <c r="A1716" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B1716" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C1716" s="1" t="n">
         <v>39299</v>
@@ -55023,24 +55023,24 @@
         </is>
       </c>
       <c r="E1716" s="1" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="F1716" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1717" customHeight="1" ht="20">
       <c r="A1717" s="1" t="n">
-        <v>1598892</v>
+        <v>1523488</v>
       </c>
       <c r="B1717" s="1" t="n">
-        <v>27486</v>
+        <v>24896</v>
       </c>
       <c r="C1717" s="1" t="n">
         <v>39347</v>
@@ -55055,24 +55055,24 @@
         </is>
       </c>
       <c r="E1717" s="1" t="n">
-        <v>30000</v>
+        <v>10000</v>
       </c>
       <c r="F1717" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">26/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1718" customHeight="1" ht="20">
       <c r="A1718" s="1" t="n">
-        <v>1523488</v>
+        <v>1598892</v>
       </c>
       <c r="B1718" s="1" t="n">
-        <v>24896</v>
+        <v>27486</v>
       </c>
       <c r="C1718" s="1" t="n">
         <v>39347</v>
@@ -55087,14 +55087,14 @@
         </is>
       </c>
       <c r="E1718" s="1" t="n">
-        <v>10000</v>
+        <v>30000</v>
       </c>
       <c r="F1718" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">26/10/2026</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
@@ -55293,10 +55293,10 @@
     </row>
     <row r="1725" customHeight="1" ht="20">
       <c r="A1725" s="1" t="n">
-        <v>1630636</v>
+        <v>1598892</v>
       </c>
       <c r="B1725" s="1" t="n">
-        <v>29656</v>
+        <v>27486</v>
       </c>
       <c r="C1725" s="1" t="n">
         <v>39296</v>
@@ -55311,24 +55311,24 @@
         </is>
       </c>
       <c r="E1725" s="1" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="F1725" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1726" customHeight="1" ht="20">
       <c r="A1726" s="1" t="n">
-        <v>1598892</v>
+        <v>1630636</v>
       </c>
       <c r="B1726" s="1" t="n">
-        <v>27486</v>
+        <v>29656</v>
       </c>
       <c r="C1726" s="1" t="n">
         <v>39296</v>
@@ -55343,24 +55343,24 @@
         </is>
       </c>
       <c r="E1726" s="1" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="F1726" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1727" customHeight="1" ht="20">
       <c r="A1727" s="1" t="n">
-        <v>1630636</v>
+        <v>1523488</v>
       </c>
       <c r="B1727" s="1" t="n">
-        <v>29656</v>
+        <v>24896</v>
       </c>
       <c r="C1727" s="1" t="n">
         <v>39300</v>
@@ -55375,24 +55375,24 @@
         </is>
       </c>
       <c r="E1727" s="1" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="F1727" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">26/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1728" customHeight="1" ht="20">
       <c r="A1728" s="1" t="n">
-        <v>1523488</v>
+        <v>1630636</v>
       </c>
       <c r="B1728" s="1" t="n">
-        <v>24896</v>
+        <v>29656</v>
       </c>
       <c r="C1728" s="1" t="n">
         <v>39300</v>
@@ -55407,14 +55407,14 @@
         </is>
       </c>
       <c r="E1728" s="1" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="F1728" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">26/10/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -57821,10 +57821,10 @@
     </row>
     <row r="1804" customHeight="1" ht="20">
       <c r="A1804" s="1" t="n">
-        <v>1598892</v>
+        <v>1523488</v>
       </c>
       <c r="B1804" s="1" t="n">
-        <v>27486</v>
+        <v>24896</v>
       </c>
       <c r="C1804" s="1" t="n">
         <v>42112</v>
@@ -57839,24 +57839,24 @@
         </is>
       </c>
       <c r="E1804" s="1" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F1804" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">26/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1805" customHeight="1" ht="20">
       <c r="A1805" s="1" t="n">
-        <v>1523488</v>
+        <v>1598892</v>
       </c>
       <c r="B1805" s="1" t="n">
-        <v>24896</v>
+        <v>27486</v>
       </c>
       <c r="C1805" s="1" t="n">
         <v>42112</v>
@@ -57871,14 +57871,14 @@
         </is>
       </c>
       <c r="E1805" s="1" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F1805" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">26/10/2026</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
@@ -59325,10 +59325,10 @@
     </row>
     <row r="1851" customHeight="1" ht="20">
       <c r="A1851" s="1" t="n">
-        <v>1630636</v>
+        <v>1523488</v>
       </c>
       <c r="B1851" s="1" t="n">
-        <v>29656</v>
+        <v>24896</v>
       </c>
       <c r="C1851" s="1" t="n">
         <v>44196</v>
@@ -59343,24 +59343,24 @@
         </is>
       </c>
       <c r="E1851" s="1" t="n">
-        <v>300</v>
+        <v>30</v>
       </c>
       <c r="F1851" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">26/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1852" customHeight="1" ht="20">
       <c r="A1852" s="1" t="n">
-        <v>1523488</v>
+        <v>1630636</v>
       </c>
       <c r="B1852" s="1" t="n">
-        <v>24896</v>
+        <v>29656</v>
       </c>
       <c r="C1852" s="1" t="n">
         <v>44196</v>
@@ -59375,14 +59375,14 @@
         </is>
       </c>
       <c r="E1852" s="1" t="n">
-        <v>30</v>
+        <v>300</v>
       </c>
       <c r="F1852" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">26/10/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -61053,10 +61053,10 @@
     </row>
     <row r="1905" customHeight="1" ht="20">
       <c r="A1905" s="1" t="n">
-        <v>1630636</v>
+        <v>1523488</v>
       </c>
       <c r="B1905" s="1" t="n">
-        <v>29656</v>
+        <v>24896</v>
       </c>
       <c r="C1905" s="1" t="n">
         <v>44199</v>
@@ -61071,24 +61071,24 @@
         </is>
       </c>
       <c r="E1905" s="1" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="F1905" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">26/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1906" customHeight="1" ht="20">
       <c r="A1906" s="1" t="n">
-        <v>1523488</v>
+        <v>1630636</v>
       </c>
       <c r="B1906" s="1" t="n">
-        <v>24896</v>
+        <v>29656</v>
       </c>
       <c r="C1906" s="1" t="n">
         <v>44199</v>
@@ -61103,14 +61103,14 @@
         </is>
       </c>
       <c r="E1906" s="1" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="F1906" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">26/10/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>

</xml_diff>

<commit_message>
Atualiza compras pendentes 25/10/2026 22:01
</commit_message>
<xml_diff>
--- a/data/COMPRAS_PENDENTES.xlsx
+++ b/data/COMPRAS_PENDENTES.xlsx
@@ -19485,10 +19485,10 @@
     </row>
     <row r="606" customHeight="1" ht="20">
       <c r="A606" s="1" t="n">
-        <v>1630636</v>
+        <v>1523488</v>
       </c>
       <c r="B606" s="1" t="n">
-        <v>29656</v>
+        <v>24896</v>
       </c>
       <c r="C606" s="1" t="n">
         <v>14161</v>
@@ -19510,17 +19510,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">30/01/2027</t>
+            <t xml:space="preserve">26/10/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="607" customHeight="1" ht="20">
       <c r="A607" s="1" t="n">
-        <v>1523488</v>
+        <v>1630636</v>
       </c>
       <c r="B607" s="1" t="n">
-        <v>24896</v>
+        <v>29656</v>
       </c>
       <c r="C607" s="1" t="n">
         <v>14161</v>
@@ -19542,7 +19542,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">26/10/2026</t>
+            <t xml:space="preserve">30/01/2027</t>
           </r>
         </is>
       </c>
@@ -21981,10 +21981,10 @@
     </row>
     <row r="684" customHeight="1" ht="20">
       <c r="A684" s="1" t="n">
-        <v>1598892</v>
+        <v>1635939</v>
       </c>
       <c r="B684" s="1" t="n">
-        <v>27486</v>
+        <v>29609</v>
       </c>
       <c r="C684" s="1" t="n">
         <v>14137</v>
@@ -21999,24 +21999,24 @@
         </is>
       </c>
       <c r="E684" s="1" t="n">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="F684" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">10/12/2026</t>
+            <t xml:space="preserve">13/11/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="685" customHeight="1" ht="20">
       <c r="A685" s="1" t="n">
-        <v>1635939</v>
+        <v>1598892</v>
       </c>
       <c r="B685" s="1" t="n">
-        <v>29609</v>
+        <v>27486</v>
       </c>
       <c r="C685" s="1" t="n">
         <v>14137</v>
@@ -22031,14 +22031,14 @@
         </is>
       </c>
       <c r="E685" s="1" t="n">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="F685" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">13/11/2026</t>
+            <t xml:space="preserve">10/12/2026</t>
           </r>
         </is>
       </c>
@@ -40829,10 +40829,10 @@
     </row>
     <row r="1273" customHeight="1" ht="20">
       <c r="A1273" s="1" t="n">
-        <v>1633775</v>
+        <v>1625869</v>
       </c>
       <c r="B1273" s="1" t="n">
-        <v>29593</v>
+        <v>43</v>
       </c>
       <c r="C1273" s="1" t="n">
         <v>30716</v>
@@ -40847,24 +40847,24 @@
         </is>
       </c>
       <c r="E1273" s="1" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="F1273" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">04/02/2027</t>
+            <t xml:space="preserve">26/01/2027</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1274" customHeight="1" ht="20">
       <c r="A1274" s="1" t="n">
-        <v>1625869</v>
+        <v>1633775</v>
       </c>
       <c r="B1274" s="1" t="n">
-        <v>43</v>
+        <v>29593</v>
       </c>
       <c r="C1274" s="1" t="n">
         <v>30716</v>
@@ -40879,24 +40879,24 @@
         </is>
       </c>
       <c r="E1274" s="1" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="F1274" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">26/01/2027</t>
+            <t xml:space="preserve">04/02/2027</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1275" customHeight="1" ht="20">
       <c r="A1275" s="1" t="n">
-        <v>1633775</v>
+        <v>1625869</v>
       </c>
       <c r="B1275" s="1" t="n">
-        <v>29593</v>
+        <v>43</v>
       </c>
       <c r="C1275" s="1" t="n">
         <v>30717</v>
@@ -40918,17 +40918,17 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">04/02/2027</t>
+            <t xml:space="preserve">26/01/2027</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1276" customHeight="1" ht="20">
       <c r="A1276" s="1" t="n">
-        <v>1625869</v>
+        <v>1633775</v>
       </c>
       <c r="B1276" s="1" t="n">
-        <v>43</v>
+        <v>29593</v>
       </c>
       <c r="C1276" s="1" t="n">
         <v>30717</v>
@@ -40950,7 +40950,7 @@
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">26/01/2027</t>
+            <t xml:space="preserve">04/02/2027</t>
           </r>
         </is>
       </c>
@@ -48733,10 +48733,10 @@
     </row>
     <row r="1520" customHeight="1" ht="20">
       <c r="A1520" s="1" t="n">
-        <v>1470722</v>
+        <v>1638359</v>
       </c>
       <c r="B1520" s="1" t="n">
-        <v>24616</v>
+        <v>29613</v>
       </c>
       <c r="C1520" s="1" t="n">
         <v>32670</v>
@@ -48751,24 +48751,24 @@
         </is>
       </c>
       <c r="E1520" s="1" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F1520" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">27/10/2026</t>
+            <t xml:space="preserve">18/11/2026</t>
           </r>
         </is>
       </c>
     </row>
     <row r="1521" customHeight="1" ht="20">
       <c r="A1521" s="1" t="n">
-        <v>1638359</v>
+        <v>1470722</v>
       </c>
       <c r="B1521" s="1" t="n">
-        <v>29613</v>
+        <v>24616</v>
       </c>
       <c r="C1521" s="1" t="n">
         <v>32670</v>
@@ -48783,14 +48783,14 @@
         </is>
       </c>
       <c r="E1521" s="1" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F1521" s="1" t="inlineStr">
         <is>
           <r>
             <rPr>
        </rPr>
-            <t xml:space="preserve">18/11/2026</t>
+            <t xml:space="preserve">27/10/2026</t>
           </r>
         </is>
       </c>

</xml_diff>